<commit_message>
Record confirmed scope in JV exclusion workbook notes
All five JVs confirmed for upload as negatives; Keolis Downer JV (Rail
Services Victoria) confirmed as staying in revenue per the "FY26 JV Rev"
source sheet definition. Also notes the BIA Location Ref (RSV175-1) as a
point to confirm with the Envizi admin when reopening the closed JV
locations. Upload rows are unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016AQN7RksV9zRGxh9oFzF9f
</commit_message>
<xml_diff>
--- a/Account_Setup_and_Data_Load_-_PM&C_JVREVJUL25toJUN26_Setup.xlsx
+++ b/Account_Setup_and_Data_Load_-_PM&C_JVREVJUL25toJUN26_Setup.xlsx
@@ -5788,7 +5788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -6282,7 +6282,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>4. Coverage — please confirm before loading: of the five JVs, only BIA currently appears as a revenue line in the loaded FY26 figures (Account_Setup_and_Data_Load_-_PM&amp;C_REVJUL25toJUN26_Setup.xlsx, and the "FY26 Rev" detail). Allied Asphalt, EDI Rail-Bombardier Transportation, Emulco and Isaac Asphalt do not appear in those revenue figures at all, so posting negatives for them reduces reported revenue by amounts that were never included (FY26: BIA 69.9 of the 128.4 total; the other four total 58.5: Allied Asphalt 11.6, EDI Rail-Bombardier 35.6, Emulco 4.2, Isaac Asphalt 7.1).</t>
+          <t>4. Coverage — CONFIRMED 4 Aug 26: all five JVs are to be uploaded as negatives. For reference: of the five, only BIA appears as a revenue line in the loaded FY26 figures (Account_Setup_and_Data_Load_-_PM&amp;C_REVJUL25toJUN26_Setup.xlsx, and the "FY26 Rev" detail); Allied Asphalt, EDI Rail-Bombardier Transportation, Emulco and Isaac Asphalt do not appear in those figures, so their negatives reduce reported revenue by amounts not previously included (FY26: BIA 69.9 of the 128.4 total; the other four total 58.5: Allied Asphalt 11.6, EDI Rail-Bombardier 35.6, Emulco 4.2, Isaac Asphalt 7.1).</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6296,14 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>5. Also note: "Rail Services Victoria Pty Ltd" (Keolis Downer JV) IS in the loaded FY26 revenue figures under REV_Keolis Downer JV (FY26 total 27.3), but is not listed on the "FY26 JV Rev" source sheet, so it is not excluded by this file. Confirm whether it should be.</t>
+          <t>5. Keolis Downer JV — CONFIRMED 4 Aug 26: not excluded. "Rail Services Victoria Pty Ltd" IS in the loaded FY26 revenue figures under REV_Keolis Downer JV (FY26 total 27.3) but is not on the "FY26 JV Rev" source sheet; the source sheet is the agreed definition of JV revenue to exclude, so it stays in revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>6. BIA Location Ref: the extract shows Location Ref "RSV175-1" for _CLOSED_REV_BIA, which looks like a Rail Services Victoria code. Copied faithfully from the extract; worth confirming with the Envizi admin when reopening the locations.</t>
         </is>
       </c>
     </row>

</xml_diff>